<commit_message>
QABUL - 2026 shabloni, AI tarjima va talaba kartasida .docx biriktirish
- QABUL - 2026: "Jami" sahifasida A ustunda guruh, shablon fayllari va
  istisnolar yangilandi (generate_qabul_shablon.py, qabul.ts, excel.ts)
- AI tarjima (/api/ai-translate, lib/qabul-ai.ts): qoidalar tanimagan muassasa
  nomlari — rasmiy o'zbekcha -> ruscha -> inglizcha; natija brauzerda keshlanadi
- Talaba kartasi: shartnoma .docx zonasi (upload_and_attach_to_student)
- AI tahlil faqat tugma bosilganda ishlaydi (.docx tashlanganda avtomatik emas)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hisobotlar/qabul/guruhlar/QABUL - 2026 (26-03).xlsx
+++ b/hisobotlar/qabul/guruhlar/QABUL - 2026 (26-03).xlsx
@@ -47,7 +47,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -57,11 +57,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8EEF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,9 +101,6 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -721,21 +713,25 @@
         <v>917090876</v>
       </c>
       <c r="F6" s="4" t="n"/>
-      <c r="G6" s="7" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
       <c r="H6" s="5" t="n"/>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>25-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Yakkabog' tumani 25-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>General Secondary School No. 25</t>
+          <t>General Secondary School No. 25, Yakkabog District</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Общеобразовательная школа №25</t>
+          <t>Общеобразовательная школа №25 Яккабагского района</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -777,21 +773,25 @@
         <v>997307709</v>
       </c>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="7" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>43-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Yakkabog' tumani 43-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>General Secondary School No. 43</t>
+          <t>General Secondary School No. 43, Yakkabog District</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Общеобразовательная школа №43</t>
+          <t>Общеобразовательная школа №43 Яккабагского района</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -1687,21 +1687,25 @@
       </c>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
-      <c r="G22" s="7" t="n"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
       <c r="H22" s="5" t="n"/>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>81-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Yakkabog' tumani 81-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>General Secondary School No. 81</t>
+          <t>General Secondary School No. 81, Yakkabog District</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>Общеобразовательная школа №81</t>
+          <t>Общеобразовательная школа №81 Яккабагского района</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -1869,21 +1873,25 @@
       <c r="F25" s="4" t="n">
         <v>880037679</v>
       </c>
-      <c r="G25" s="7" t="n"/>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
       <c r="H25" s="5" t="n"/>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>69-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Yakkabog' tumani 69-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>General Secondary School No. 69</t>
+          <t>General Secondary School No. 69, Yakkabog District</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Общеобразовательная школа №69</t>
+          <t>Общеобразовательная школа №69 Яккабагского района</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2415,21 +2423,25 @@
         <v>997422473</v>
       </c>
       <c r="F34" s="4" t="n"/>
-      <c r="G34" s="7" t="n"/>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
       <c r="H34" s="5" t="n"/>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>69-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Yakkabog' tumani 69-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>General Secondary School No. 69</t>
+          <t>General Secondary School No. 69, Yakkabog District</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>Общеобразовательная школа №69</t>
+          <t>Общеобразовательная школа №69 Яккабагского района</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
@@ -2535,21 +2547,25 @@
       <c r="F36" s="4" t="n">
         <v>912162304</v>
       </c>
-      <c r="G36" s="7" t="n"/>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Qashqadaryo, Yakkabog' tumani</t>
+        </is>
+      </c>
       <c r="H36" s="5" t="n"/>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>4-sonli umumiy o'rta ta'lim maktabi</t>
+          <t>Yakkabog' tumani 4-sonli umumiy o'rta ta'lim maktabi</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>General Secondary School No. 4</t>
+          <t>General Secondary School No. 4, Yakkabog District</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>Общеобразовательная школа №4</t>
+          <t>Общеобразовательная школа №4 Яккабагского района</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">

</xml_diff>